<commit_message>
Add full Cochrane CENTRAL bibliographic data and Library links
Replace the shortened working titles for the 10 Cochrane CENTRAL
records with their real titles, authors/trial registry IDs, journal
citations, and direct Cochrane Library links, as provided by the PI.

Screening_AO_Spine.xlsx: the Cochrane sheet now shows authors,
source citation, and a clickable link per record (no abstract was
available, so this lets reviewers open the record directly).
screening_tracking_template.csv: same data, plus a url column.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QefD8iXX1bH7VELxycXejs
</commit_message>
<xml_diff>
--- a/screening/Screening_AO_Spine.xlsx
+++ b/screening/Screening_AO_Spine.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,6 +53,12 @@
       <i val="1"/>
       <color rgb="00C0392B"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001155CC"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -105,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -122,8 +128,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -136,6 +142,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -541,7 +550,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2. Para cada fila, leé el título y el resumen, y marcá una decisión en la columna "Decisión": Include, Exclude o Maybe.</t>
+          <t>2. Para cada fila, leé el título y el resumen (o abrí el link a Cochrane Library en la hoja de Cochrane), y marcá una decisión en la columna "Decisión": Include, Exclude o Maybe.</t>
         </is>
       </c>
     </row>
@@ -569,7 +578,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>6. Los 10 registros de Cochrane CENTRAL NO están en Rayyan (no se pudieron importar por incompatibilidad de formato) — este Excel es la única vía para revisarlos por ahora. No tienen resumen cargado; si necesitás el abstract completo, buscá el título en Cochrane Library.</t>
+          <t>6. Los 10 registros de Cochrane CENTRAL NO están en Rayyan (no se pudieron importar por incompatibilidad de formato). Esta hoja tiene el título, autores/registro, revista y un link directo a Cochrane Library para leer el resumen completo ahí.</t>
         </is>
       </c>
     </row>
@@ -833,19 +842,19 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF('Screening 10 (Cochrane)'!C3:C12,"Include")</f>
+        <f>COUNTIF('Screening 10 (Cochrane)'!G3:G12,"Include")</f>
         <v/>
       </c>
       <c r="C5" s="7">
-        <f>COUNTIF('Screening 10 (Cochrane)'!C3:C12,"Exclude")</f>
+        <f>COUNTIF('Screening 10 (Cochrane)'!G3:G12,"Exclude")</f>
         <v/>
       </c>
       <c r="D5" s="7">
-        <f>COUNTIF('Screening 10 (Cochrane)'!C3:C12,"Maybe")</f>
+        <f>COUNTIF('Screening 10 (Cochrane)'!G3:G12,"Maybe")</f>
         <v/>
       </c>
       <c r="E5" s="7">
-        <f>10-COUNTA('Screening 10 (Cochrane)'!C3:C12)</f>
+        <f>10-COUNTA('Screening 10 (Cochrane)'!G3:G12)</f>
         <v/>
       </c>
     </row>
@@ -2021,19 +2030,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>Estos 10 registros no están en Rayyan (no se pudieron importar). No tienen resumen cargado — buscar el título en Cochrane Library si hace falta el abstract completo.</t>
+          <t>Estos 10 registros no están en Rayyan (no se pudieron importar). Hacé click en el título para abrir el resumen completo en Cochrane Library.</t>
         </is>
       </c>
     </row>
@@ -2045,15 +2058,35 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>Título</t>
+          <t>Título (click para abrir en Cochrane Library)</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
+          <t>Autores / Registro</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>Revista / fuente</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>Año</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>Base de origen</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
           <t>Decisión</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="H2" s="10" t="inlineStr">
         <is>
           <t>Motivo</t>
         </is>
@@ -2065,13 +2098,33 @@
           <t>COCH-01</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
-        <is>
-          <t>TLICS in thoracolumbar fractures — 2023 Türkiye earthquake</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="inlineStr"/>
-      <c r="D3" s="12" t="inlineStr"/>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>Management of Thoracolumbar Injury Classification and Severity Score (TLICS) 4 thoracolumbar fractures after natural disasters: comparative outcomes of conservative and surgical treatments following the 2023 Türkiye earthquake</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>H Gok, A Emet, NB Odabasi, A Daylak, E Akgun, ME Emrahoglu, B Abbasoglu, H Dolgun</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Turkish journal of trauma &amp; emergency surgery, 2025, 31(9), 907-912</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>CINAHL</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr"/>
+      <c r="H3" s="12" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -2079,13 +2132,29 @@
           <t>COCH-02</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
-        <is>
-          <t>Preoperative Postural Reduction vs Intraoperative Distraction — AO A3/A4</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr"/>
-      <c r="D4" s="12" t="inlineStr"/>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Comparison of Preoperative Postural Reduction versus Intraoperative Distraction Reduction on Radiographic and Clinical Outcomes in Posterior Short-Segment Fixation for AO A3/A4 Thoracolumbar Fractures</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr"/>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Registro ChiCTR2600128437 — https://trialsearch.who.int/Trial2.aspx?TrialID=ChiCTR2600128437</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>ICTRP</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr"/>
+      <c r="H4" s="12" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -2093,13 +2162,33 @@
           <t>COCH-03</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>Intermediate screw in thoracolumbar fracture fixation</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr"/>
-      <c r="D5" s="12" t="inlineStr"/>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Could intermediate screw in thoracolumbar fracture fixation save motion levels? comparative study between long segment and short segment with intermediate screw fixation</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>T El Hewala, A El-Adawy, M Hussein</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Global spine journal, 2017, 7(2), 53S</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Embase</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr"/>
+      <c r="H5" s="12" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -2107,13 +2196,33 @@
           <t>COCH-04</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Percutaneous vs Conventional Spinal Fixation</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr"/>
-      <c r="D6" s="12" t="inlineStr"/>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Outcomes of Percutaneous Fixation in Thoracolumbar Fractures v/s Conventional Spinal Fixation</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>A Pandey, S Beedkar, S Jain</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>International journal of current pharmaceutical review and research, 2026, 18(3), 1411-1414</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Embase</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr"/>
+      <c r="H6" s="12" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -2121,13 +2230,33 @@
           <t>COCH-05</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>Mono-axial vs Poly-axial pedicle screw</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr"/>
-      <c r="D7" s="12" t="inlineStr"/>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>P572: mono-axial versus poly-axial pedicle screw fixation for thoraco-lumbar fractures: a randomised controlled trial</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>AS Abdelgawaad, IA El-Hameed, M Ibrahim, A Hassan, M El-Meshwawy</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Global spine journal, 2023, 13(2), 511S</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Embase</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr"/>
+      <c r="H7" s="12" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -2135,13 +2264,33 @@
           <t>COCH-06</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>Percutaneous fixation — index level fixation</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr"/>
-      <c r="D8" s="12" t="inlineStr"/>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Percutaneous fixation of thoracolumbar fractures. Does index level fixation help in fracture reduction and stability?</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>T ElHewala, A El-Adawy</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Global spine journal, 2018, 8(1), 364S</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Embase</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr"/>
+      <c r="H8" s="12" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
@@ -2149,13 +2298,33 @@
           <t>COCH-07</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>Erector spinae plane block — analgesia post cirugía</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr"/>
-      <c r="D9" s="12" t="inlineStr"/>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>A355: does erector spinae plane block decrease amount of analgesia needed after minimal-invasive posterior transpedicular stabilization in patient with vertebral body fracture? A prospective double-blinded controlled study</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>M Holas, J Hlasny, R Gajdos, M Venglarcik, J Svac, T Hrin, M Botka, R Nagypal, T Pucan, K Schnake, P Merjavy, S Wimmerova</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Global spine journal, 2022, 12(3), 200S-201S</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>Embase</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr"/>
+      <c r="H9" s="12" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
@@ -2163,13 +2332,29 @@
           <t>COCH-08</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>Riluzole and Methylprednisolone in spinal cord injury</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr"/>
-      <c r="D10" s="12" t="inlineStr"/>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Effect of Riluzole and Methylprednisolone in spina cord injury</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr"/>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Registro IRCT20240722062515N1 — https://trialsearch.who.int/Trial2.aspx?TrialID=IRCT20240722062515N1</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>ICTRP</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr"/>
+      <c r="H10" s="12" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -2177,13 +2362,29 @@
           <t>COCH-09</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>Orthosis in Cervical Spine Fracture Treatment</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr"/>
-      <c r="D11" s="12" t="inlineStr"/>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Study on Orthosis in Cervical Spine Fracture Treatment</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr"/>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Registro NCT06848660 — https://clinicaltrials.gov/study/NCT06848660</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>CT.gov</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr"/>
+      <c r="H11" s="12" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
@@ -2191,23 +2392,55 @@
           <t>COCH-10</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>Direct Decompression for Thoracolumbar Burst Fractures with Neurological Compromise</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr"/>
-      <c r="D12" s="12" t="inlineStr"/>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Necessity of Direct Decompression for Thoracolumbar Junction Burst Fractures with Neurological Compromise</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>NK Jaiswal, V Kumar, V Puvanesarajah, A Dagar, M Prakash, M Dhillon, SS Dhatt</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>World neurosurgery, 2020, 142, e413-e419</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>PubMed+Embase</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr"/>
+      <c r="H12" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C3 C4 C5 C6 C7 C8 C9 C10 C11 C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G3 G4 G5 G6 G7 G8 G9 G10 G11 G12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Include,Exclude,Maybe"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId10"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>